<commit_message>
Atualizacao da interface, mixagem e novas imagens
</commit_message>
<xml_diff>
--- a/app_estudo_havayanas/www/ritmos.xlsx
+++ b/app_estudo_havayanas/www/ritmos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alvaroferreira/Downloads/app_estudo_havayanas/www/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8242b9476157fafd/Aplicativos_Shiny/projeto_havayanas/app_estudo_havayanas/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399CEAB1-49B8-BF4A-B210-06DC92F2808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{399CEAB1-49B8-BF4A-B210-06DC92F2808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F6C3C7B-5BE5-3C4C-A0BE-51BACA327EC4}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-8640" yWindow="-28200" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="levadas" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">convencoes!$A$1:$F$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">levadas!$A$1:$E$137</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="149">
   <si>
     <t>Levada</t>
   </si>
@@ -482,6 +482,9 @@
   </si>
   <si>
     <t>pe*</t>
+  </si>
+  <si>
+    <t>Alvaro</t>
   </si>
 </sst>
 </file>
@@ -815,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -2799,6 +2802,20 @@
         <v>139</v>
       </c>
       <c r="D137" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
+        <v>148</v>
+      </c>
+      <c r="B138" t="s">
+        <v>9</v>
+      </c>
+      <c r="C138" t="s">
+        <v>139</v>
+      </c>
+      <c r="D138" t="s">
         <v>139</v>
       </c>
     </row>

</xml_diff>